<commit_message>
made single code to multiple codes
</commit_message>
<xml_diff>
--- a/log_data.xlsx
+++ b/log_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -662,7 +662,1329 @@
           <t>23:10:11</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>23:25:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>45465</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>23:26:01</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>23:26:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="n">
+        <v>112201035</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Malaka Kishore</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>45467</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>19:43:55</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>19:48:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>45467</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>19:43:43</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>20:06:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>45472</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>23:33:45</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>23:33:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>142201005</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dadi Rishitha</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>45467</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>20:06:51</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>142201008</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mogili Lavanya</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>45467</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>20:07:11</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>112201035</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Malaka Kishore</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>45468</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>12:36:35</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>45472</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>23:49:41</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>192201001</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New Person Name</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>New Department</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>08:30:00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>45472</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Sahyadri Libray</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>45472</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Sahyadri Libray</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>13:36:40</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>23:37:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Nila Library</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>23:43:33</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Nila Library</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>23:44:12</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>25</v>
+      </c>
+      <c r="B20" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UG </t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>20:57:36</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>20:59:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>26</v>
+      </c>
+      <c r="B21" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>21:01:14</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>21:13:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="n">
+        <v>142201007</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Ashwini Kannan K</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Nila Library</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>00:34:59</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="n">
+        <v>132201034</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Cheekatla Lohith</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>00:41:30</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="n">
+        <v>142201008</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mogili Lavanya</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>14:39:47</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="n">
+        <v>112201008</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Nandhana Sunil</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Sahyadri Library</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>16:40:03</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="n">
+        <v>122201006</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Konduru Bhanu Chandrika</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>UG student</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>17:10:31</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="n">
+        <v>102404005</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Aarathy. S.S</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>17:15:13</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>21:13:51</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>142201005</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dadi Rishitha</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>23:03:00</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>23:08:00</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>112201004</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Muluguru Pranitha</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>15:22:00</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>112201009</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Swadha Swaroop</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>15:22:00</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>15:23:00</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>112101035</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PARMAR JIGNESH JAYANTIBHAI</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>15:23:00</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>

</xml_diff>

<commit_message>
final code is ready
</commit_message>
<xml_diff>
--- a/log_data.xlsx
+++ b/log_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1858,7 +1858,11 @@
           <t>15:22:00</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1900,7 +1904,11 @@
           <t>15:22:00</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1942,7 +1950,11 @@
           <t>15:23:00</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1984,7 +1996,1705 @@
           <t>15:23:00</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>102201002</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ramavath Bhadra</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>23:33:00</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>36</v>
+      </c>
+      <c r="B36" t="n">
+        <v>112201006</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sangam</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>15:17:00</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>15:17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>15:11:00</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>15:21:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>122101011</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GARIMA RANJAN</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>17:47:00</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>122101048</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SHRI GOKUL K</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>17:48:00</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>132101012</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ISHIKA GUPTA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>17:48:00</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>112201011</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Maloth Sony</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>17:48:00</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>112201015</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Kaushik Rawat</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>17:48:00</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>122201002</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Gayathri S</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>17:49:00</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>122201042</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Mohammed Azim</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>17:49:00</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>132201008</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Priyamvada Kaneti</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>17:49:00</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>132201029</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mouhamad Sayif</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>17:49:00</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>142201006</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Salveru Jayati</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>17:50:00</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>142201018</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Jadhav Akshay Sanjay</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>17:50:00</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>102301031</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Savula Vaishnavi</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>17:50:00</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>132301019</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Karreddula Rahul</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>17:50:00</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>142301021</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Maram Ruthvi</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>17:51:00</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>142301023</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Medepalli Julekhya</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>17:51:00</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>142301025</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Mudduluru Thanish Kumar Raju</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>17:51:00</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>112301022</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Mocharla Sai Akash</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>17:51:00</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>102004005</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>MITHULRAJ M</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>17:53:00</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>102114008</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Vismaya K</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>17:53:00</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>102204002</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Jayakrishnan Puthiya Veettil</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>17:54:00</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>112114006</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bijin Elsa Baby</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>17:54:00</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>122004003</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ATHUL O ASOK</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>17:54:00</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>122004004</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AYYAPPADAS.R</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>17:54:00</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>122204004</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>THOUFEER K K</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>17:54:00</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>162404003</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Jadeera Aboobaker</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ESSENCE</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>17:55:00</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>132004001</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ARUN KRISHNAN  K S</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Research Scholar</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>17:55:00</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>45477</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>11:16:00</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>45477</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>11:16:00</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>142201008</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Mogili Lavanya</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>45477</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>11:16:00</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>67</v>
+      </c>
+      <c r="B67" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>13:44:00</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>14:02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>68</v>
+      </c>
+      <c r="B68" t="n">
+        <v>112201035</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Malaka Kishore</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>14:02:00</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>13:43:00</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>14:16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>14:18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Nila</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>14:18:00</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>

</xml_diff>

<commit_message>
add memeber button was added
</commit_message>
<xml_diff>
--- a/log_data.xlsx
+++ b/log_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3836,7 +3836,375 @@
           <t>16:10:00</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>16:19:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>75</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1429</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>76</v>
+      </c>
+      <c r="B76" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>17:05:00</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>17:05:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>77</v>
+      </c>
+      <c r="B77" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>17:08:00</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>17:08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Dr. Frank Green</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>faculty</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>45479</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>16:47:00</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>142201003</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Ganedi Satya Harika</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Data Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>45482</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>45482</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>12:24:00</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>45484</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>11:29:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="n">
+        <v>112201044</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Kallepally Sai Kiran</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>45484</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Sahyadri</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>12:12:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>

</xml_diff>